<commit_message>
feat: update passive items balance tools and food skills
</commit_message>
<xml_diff>
--- a/GourmetProject/GameConfig/Datas/action.xlsx
+++ b/GourmetProject/GameConfig/Datas/action.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="action" sheetId="1" r:id="R6c6bc2a6c2494778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="large_group" sheetId="2" r:id="Rb6723b9641f74f05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="small_group" sheetId="3" r:id="Re0af9eb9d24f43e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="action" sheetId="1" r:id="R88c3276b39d4456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="large_group" sheetId="2" r:id="R81e1915cfcfc436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="small_group" sheetId="3" r:id="R8c7627cfb6a04fe2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -284,9 +284,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">偿还高利贷</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">扣除400金币</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Effect</x:t>
@@ -3570,17 +3567,17 @@
       <x:c r="C20" s="1" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D20" s="1" t="s">
+      <x:c r="D20" s="1" t="str">
+        <x:v>扣除200金币</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="E20" s="1" t="s">
+      <x:c r="G20" s="1" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="G20" s="1" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="H20" s="1">
-        <x:v>-400</x:v>
+      <x:c r="H20" s="1" t="n">
+        <x:v>-200</x:v>
       </x:c>
       <x:c r="I20"/>
       <x:c r="J20" s="1">
@@ -3594,19 +3591,19 @@
     </x:row>
     <x:row r="21">
       <x:c r="B21" s="1" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="s">
+      <x:c r="D21" s="1" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="D21" s="1" t="s">
+      <x:c r="E21" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="G21" s="1" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="E21" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="G21" s="1" t="s">
-        <x:v>97</x:v>
       </x:c>
       <x:c r="H21" s="1">
         <x:v>0</x:v>
@@ -3661,16 +3658,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="s">
+      <x:c r="F1" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="F1" t="s">
-        <x:v>100</x:v>
-      </x:c>
       <x:c r="G1" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H1" s="1"/>
       <x:c r="I1"/>
@@ -3687,22 +3684,22 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="D2" s="1" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="D2" s="1" t="s">
+      <x:c r="E2" s="1" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="s">
+      <x:c r="F2" s="1" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="s">
+      <x:c r="G2" s="1" t="s">
         <x:v>106</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>107</x:v>
       </x:c>
       <x:c r="H2" s="1"/>
       <x:c r="I2"/>
@@ -3725,16 +3722,16 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="D3" s="1" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="E3" s="1" t="s">
+      <x:c r="F3" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="G3" t="s">
         <x:v>109</x:v>
-      </x:c>
-      <x:c r="F3" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="G3" t="s">
-        <x:v>110</x:v>
       </x:c>
       <x:c r="H3" s="1"/>
       <x:c r="I3"/>
@@ -3748,22 +3745,22 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1">
       <x:c r="B4" s="1" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="C4" s="1" t="s">
-        <x:v>112</x:v>
       </x:c>
       <x:c r="D4">
         <x:v>400</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="F4" s="2" t="s">
+      <x:c r="G4" s="2" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="G4" s="2" t="s">
-        <x:v>115</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:f>""</x:f>
@@ -3850,22 +3847,22 @@
     </x:row>
     <x:row r="8" s="1" customFormat="1">
       <x:c r="B8" s="1" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
         <x:v>116</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>117</x:v>
       </x:c>
       <x:c r="D8">
         <x:v>200</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="F8" s="2" t="s">
+      <x:c r="G8" s="2" t="s">
         <x:v>119</x:v>
-      </x:c>
-      <x:c r="G8" s="2" t="s">
-        <x:v>120</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:f>""</x:f>
@@ -3952,22 +3949,22 @@
     </x:row>
     <x:row r="12" s="1" customFormat="1">
       <x:c r="B12" s="1" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="C12" s="1" t="s">
+      <x:c r="D12">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="D12">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E12" s="2" t="s">
+      <x:c r="F12" s="2" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="s">
+      <x:c r="G12" s="2" t="s">
         <x:v>124</x:v>
-      </x:c>
-      <x:c r="G12" s="2" t="s">
-        <x:v>125</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
         <x:f>""</x:f>
@@ -4055,22 +4052,22 @@
     </x:row>
     <x:row r="16" s="1" customFormat="1">
       <x:c r="B16" s="1" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="C16" s="1" t="s">
+      <x:c r="D16">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="G16" s="2" t="s">
         <x:v>127</x:v>
-      </x:c>
-      <x:c r="D16">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E16" s="2" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="F16" s="2" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="G16" s="2" t="s">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
         <x:f>""</x:f>
@@ -4158,22 +4155,22 @@
     </x:row>
     <x:row r="20" s="1" customFormat="1">
       <x:c r="B20" s="1" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="s">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="C20" s="1" t="s">
-        <x:v>130</x:v>
       </x:c>
       <x:c r="D20">
         <x:v>150</x:v>
       </x:c>
       <x:c r="E20" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F20" s="2" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="G20" s="2" t="s">
-        <x:v>131</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
         <x:f>""</x:f>
@@ -4260,22 +4257,22 @@
     </x:row>
     <x:row r="24" s="1" customFormat="1">
       <x:c r="B24" s="1" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="C24" s="1" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="C24" s="1" t="s">
+      <x:c r="D24">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="G24" s="2" t="s">
         <x:v>133</x:v>
-      </x:c>
-      <x:c r="D24">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E24" s="2" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="F24" s="2" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="G24" s="2" t="s">
-        <x:v>134</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
         <x:f>""</x:f>
@@ -4362,22 +4359,22 @@
     </x:row>
     <x:row r="28" s="1" customFormat="1">
       <x:c r="B28" s="1" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="C28" s="1" t="s">
         <x:v>135</x:v>
-      </x:c>
-      <x:c r="C28" s="1" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="D28">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E28" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F28" s="2" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="G28" s="2" t="s">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
         <x:f>""</x:f>
@@ -4553,10 +4550,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="s">
-        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1">
@@ -4564,16 +4561,16 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="D2" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="D2" s="1" t="s">
+      <x:c r="E2" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1">
@@ -4590,316 +4587,316 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1">
       <x:c r="B4" s="1" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="C4" s="1" t="s">
+      <x:c r="D4" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="s">
         <x:v>145</x:v>
-      </x:c>
-      <x:c r="D4" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E4" s="1" t="s">
-        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1">
       <x:c r="B5" s="1" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C5" s="1" t="s">
+      <x:c r="D5" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="D5" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E5" s="1" t="s">
+      <x:c r="R5" s="1" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="R5" s="1" t="s">
-        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1">
       <x:c r="B6" s="1" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="C6" s="1" t="s">
+      <x:c r="D6" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="D6" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E6" s="1" t="s">
+      <x:c r="R6" s="1" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="R6" s="1" t="s">
-        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1">
       <x:c r="B7" s="1" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="C7" s="1" t="s">
+      <x:c r="D7" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="D7" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
+      <x:c r="R7" s="1" t="s">
         <x:v>157</x:v>
-      </x:c>
-      <x:c r="R7" s="1" t="s">
-        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1">
       <x:c r="B8" s="1" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="C8" s="1" t="s">
+      <x:c r="D8" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="D8" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E8" s="1" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1">
       <x:c r="B9" s="1" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="C9" s="1" t="s">
+      <x:c r="D9" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="s">
         <x:v>163</x:v>
-      </x:c>
-      <x:c r="D9" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E9" s="1" t="s">
-        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1">
       <x:c r="B10" s="1" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="C10" s="1" t="s">
+      <x:c r="D10" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="D10" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E10" s="1" t="s">
-        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1">
       <x:c r="B11" s="1" t="s">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="C11" s="1" t="s">
+      <x:c r="D11" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E11" s="1" t="s">
         <x:v>169</x:v>
-      </x:c>
-      <x:c r="D11" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E11" s="1" t="s">
-        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="1" customFormat="1">
       <x:c r="B12" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="C12" s="1" t="s">
+      <x:c r="D12" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E12" s="1" t="s">
         <x:v>172</x:v>
-      </x:c>
-      <x:c r="D12" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E12" s="1" t="s">
-        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="1" customFormat="1">
       <x:c r="B13" s="1" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="C13" s="1" t="s">
+      <x:c r="D13" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="s">
         <x:v>175</x:v>
-      </x:c>
-      <x:c r="D13" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E13" s="1" t="s">
-        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="1" customFormat="1">
       <x:c r="B14" s="1" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="C14" s="1" t="s">
+      <x:c r="D14" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="D14" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E14" s="1" t="s">
-        <x:v>179</x:v>
-      </x:c>
       <x:c r="L14" s="1" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="M14" s="1" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="M14" s="1" t="s">
-        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1">
       <x:c r="B15" s="1" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="s">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="C15" s="1" t="s">
+      <x:c r="D15" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="D15" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E15" s="1" t="s">
-        <x:v>182</x:v>
-      </x:c>
       <x:c r="L15" s="1" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="M15" s="1" t="s">
         <x:v>116</x:v>
-      </x:c>
-      <x:c r="M15" s="1" t="s">
-        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="1" customFormat="1">
       <x:c r="B16" s="1" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="C16" s="1" t="s">
+      <x:c r="D16" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="D16" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E16" s="1" t="s">
-        <x:v>185</x:v>
-      </x:c>
       <x:c r="L16" s="1" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="M16" s="1" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="M16" s="1" t="s">
-        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="1" customFormat="1">
       <x:c r="B17" s="1" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="C17" s="1" t="s">
+      <x:c r="D17" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E17" s="1" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="D17" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E17" s="1" t="s">
-        <x:v>188</x:v>
-      </x:c>
       <x:c r="L17" s="1" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="M17" s="1" t="s">
         <x:v>126</x:v>
-      </x:c>
-      <x:c r="M17" s="1" t="s">
-        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="1" customFormat="1">
       <x:c r="B18" s="1" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="C18" s="1" t="s">
+      <x:c r="D18" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E18" s="1" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="D18" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E18" s="1" t="s">
+      <x:c r="L18" s="1" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="L18" s="1" t="s">
+      <x:c r="M18" s="1" t="s">
         <x:v>192</x:v>
-      </x:c>
-      <x:c r="M18" s="1" t="s">
-        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="1" customFormat="1">
       <x:c r="B19" s="1" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="C19" s="1" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="C19" s="1" t="s">
+      <x:c r="D19" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E19" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="D19" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E19" s="1" t="s">
-        <x:v>196</x:v>
-      </x:c>
       <x:c r="L19" s="1" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="M19" s="1" t="s">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="M19" s="1" t="s">
-        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="1" customFormat="1">
       <x:c r="B20" s="1" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="s">
         <x:v>197</x:v>
       </x:c>
-      <x:c r="C20" s="1" t="s">
+      <x:c r="D20" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="D20" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E20" s="1" t="s">
+      <x:c r="L20" s="1" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="M20" s="1" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="L20" s="1" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M20" s="1" t="s">
-        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="1" customFormat="1">
       <x:c r="B21" s="1" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="s">
+      <x:c r="D21" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E21" s="1" t="s">
         <x:v>202</x:v>
       </x:c>
-      <x:c r="D21" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E21" s="1" t="s">
-        <x:v>203</x:v>
-      </x:c>
       <x:c r="L21" s="1" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="M21" s="1" t="s">
         <x:v>135</x:v>
-      </x:c>
-      <x:c r="M21" s="1" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="R21" s="1" t="s">
         <x:v>31</x:v>
@@ -4913,22 +4910,22 @@
     </x:row>
     <x:row r="22" s="1" customFormat="1">
       <x:c r="B22" s="1" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="C22" s="1" t="s">
+      <x:c r="D22" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E22" s="1" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="D22" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E22" s="1" t="s">
+      <x:c r="L22" s="1" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="L22" s="1" t="s">
+      <x:c r="M22" s="1" t="s">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="M22" s="1" t="s">
-        <x:v>208</x:v>
       </x:c>
       <x:c r="R22" s="1" t="s">
         <x:v>31</x:v>
@@ -4942,16 +4939,16 @@
     </x:row>
     <x:row r="23" s="1" customFormat="1">
       <x:c r="B23" s="1" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="C23" s="1" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="C23" s="1" t="s">
+      <x:c r="D23" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E23" s="1" t="s">
         <x:v>210</x:v>
-      </x:c>
-      <x:c r="D23" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E23" s="1" t="s">
-        <x:v>211</x:v>
       </x:c>
       <x:c r="R23" s="1" t="s">
         <x:v>31</x:v>
@@ -4965,16 +4962,16 @@
     </x:row>
     <x:row r="24" s="1" customFormat="1">
       <x:c r="B24" s="1" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="C24" s="1" t="s">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="C24" s="1" t="s">
+      <x:c r="D24" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E24" s="1" t="s">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="D24" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E24" s="1" t="s">
-        <x:v>214</x:v>
       </x:c>
       <x:c r="R24" s="1" t="s">
         <x:v>31</x:v>
@@ -4988,16 +4985,16 @@
     </x:row>
     <x:row r="25" s="1" customFormat="1">
       <x:c r="B25" s="1" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="C25" s="1" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="C25" s="1" t="s">
+      <x:c r="D25" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E25" s="1" t="s">
         <x:v>216</x:v>
-      </x:c>
-      <x:c r="D25" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E25" s="1" t="s">
-        <x:v>217</x:v>
       </x:c>
       <x:c r="R25" s="1" t="s">
         <x:v>31</x:v>
@@ -5011,16 +5008,16 @@
     </x:row>
     <x:row r="26" s="1" customFormat="1">
       <x:c r="B26" s="1" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="C26" s="1" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="C26" s="1" t="s">
+      <x:c r="D26" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E26" s="1" t="s">
         <x:v>219</x:v>
-      </x:c>
-      <x:c r="D26" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E26" s="1" t="s">
-        <x:v>220</x:v>
       </x:c>
       <x:c r="R26" s="1" t="s">
         <x:v>31</x:v>
@@ -5034,16 +5031,16 @@
     </x:row>
     <x:row r="27" s="1" customFormat="1">
       <x:c r="B27" s="1" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="C27" s="1" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="C27" s="1" t="s">
+      <x:c r="D27" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E27" s="1" t="s">
         <x:v>222</x:v>
-      </x:c>
-      <x:c r="D27" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E27" s="1" t="s">
-        <x:v>223</x:v>
       </x:c>
       <x:c r="R27" s="1" t="s">
         <x:v>38</x:v>
@@ -5057,16 +5054,16 @@
     </x:row>
     <x:row r="28" s="1" customFormat="1">
       <x:c r="B28" s="1" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="C28" s="1" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="C28" s="1" t="s">
+      <x:c r="D28" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E28" s="1" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="D28" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E28" s="1" t="s">
-        <x:v>226</x:v>
       </x:c>
       <x:c r="R28" s="1" t="s">
         <x:v>38</x:v>
@@ -5080,16 +5077,16 @@
     </x:row>
     <x:row r="29" s="1" customFormat="1">
       <x:c r="B29" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="C29" s="1" t="s">
         <x:v>227</x:v>
       </x:c>
-      <x:c r="C29" s="1" t="s">
+      <x:c r="D29" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E29" s="1" t="s">
         <x:v>228</x:v>
-      </x:c>
-      <x:c r="D29" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E29" s="1" t="s">
-        <x:v>229</x:v>
       </x:c>
       <x:c r="R29" s="1" t="s">
         <x:v>38</x:v>
@@ -5103,16 +5100,16 @@
     </x:row>
     <x:row r="30" s="1" customFormat="1">
       <x:c r="B30" s="1" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="C30" s="1" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="C30" s="1" t="s">
+      <x:c r="D30" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E30" s="1" t="s">
         <x:v>231</x:v>
-      </x:c>
-      <x:c r="D30" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E30" s="1" t="s">
-        <x:v>232</x:v>
       </x:c>
       <x:c r="R30" s="1" t="s">
         <x:v>42</x:v>
@@ -5126,16 +5123,16 @@
     </x:row>
     <x:row r="31" s="1" customFormat="1">
       <x:c r="B31" s="1" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="C31" s="1" t="s">
         <x:v>233</x:v>
       </x:c>
-      <x:c r="C31" s="1" t="s">
+      <x:c r="D31" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E31" s="1" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="D31" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E31" s="1" t="s">
-        <x:v>235</x:v>
       </x:c>
       <x:c r="R31" s="1" t="s">
         <x:v>31</x:v>
@@ -5146,16 +5143,16 @@
     </x:row>
     <x:row r="32" s="1" customFormat="1">
       <x:c r="B32" s="1" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="C32" s="1" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="C32" s="1" t="s">
+      <x:c r="D32" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E32" s="1" t="s">
         <x:v>237</x:v>
-      </x:c>
-      <x:c r="D32" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E32" s="1" t="s">
-        <x:v>238</x:v>
       </x:c>
       <x:c r="R32" s="1" t="s">
         <x:v>31</x:v>
@@ -5166,16 +5163,16 @@
     </x:row>
     <x:row r="33" s="1" customFormat="1">
       <x:c r="B33" s="1" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="C33" s="1" t="s">
         <x:v>239</x:v>
       </x:c>
-      <x:c r="C33" s="1" t="s">
+      <x:c r="D33" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E33" s="1" t="s">
         <x:v>240</x:v>
-      </x:c>
-      <x:c r="D33" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E33" s="1" t="s">
-        <x:v>241</x:v>
       </x:c>
       <x:c r="R33" s="1" t="s">
         <x:v>31</x:v>
@@ -5186,16 +5183,16 @@
     </x:row>
     <x:row r="34" s="1" customFormat="1">
       <x:c r="B34" s="1" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="C34" s="1" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="C34" s="1" t="s">
+      <x:c r="D34" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E34" s="1" t="s">
         <x:v>243</x:v>
-      </x:c>
-      <x:c r="D34" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E34" s="1" t="s">
-        <x:v>244</x:v>
       </x:c>
       <x:c r="R34" s="1" t="s">
         <x:v>31</x:v>
@@ -5206,16 +5203,16 @@
     </x:row>
     <x:row r="35" s="1" customFormat="1">
       <x:c r="B35" s="1" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C35" s="1" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="C35" s="1" t="s">
+      <x:c r="D35" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E35" s="1" t="s">
         <x:v>246</x:v>
-      </x:c>
-      <x:c r="D35" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E35" s="1" t="s">
-        <x:v>247</x:v>
       </x:c>
       <x:c r="R35" s="1" t="s">
         <x:v>38</x:v>
@@ -5226,16 +5223,16 @@
     </x:row>
     <x:row r="36" s="1" customFormat="1">
       <x:c r="B36" s="1" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="C36" s="1" t="s">
         <x:v>248</x:v>
       </x:c>
-      <x:c r="C36" s="1" t="s">
+      <x:c r="D36" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E36" s="1" t="s">
         <x:v>249</x:v>
-      </x:c>
-      <x:c r="D36" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E36" s="1" t="s">
-        <x:v>250</x:v>
       </x:c>
       <x:c r="R36" s="1" t="s">
         <x:v>38</x:v>
@@ -5246,16 +5243,16 @@
     </x:row>
     <x:row r="37" s="1" customFormat="1">
       <x:c r="B37" s="1" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C37" s="1" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="C37" s="1" t="s">
+      <x:c r="D37" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E37" s="1" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="D37" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E37" s="1" t="s">
-        <x:v>253</x:v>
       </x:c>
       <x:c r="L37" s="1" t="s">
         <x:v>31</x:v>
@@ -5269,16 +5266,16 @@
     </x:row>
     <x:row r="38" s="1" customFormat="1">
       <x:c r="B38" s="1" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="C38" s="1" t="s">
         <x:v>254</x:v>
       </x:c>
-      <x:c r="C38" s="1" t="s">
+      <x:c r="D38" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E38" s="1" t="s">
         <x:v>255</x:v>
-      </x:c>
-      <x:c r="D38" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E38" s="1" t="s">
-        <x:v>256</x:v>
       </x:c>
       <x:c r="L38" s="1" t="s">
         <x:v>38</x:v>
@@ -5292,16 +5289,16 @@
     </x:row>
     <x:row r="39" s="1" customFormat="1">
       <x:c r="B39" s="1" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="C39" s="1" t="s">
         <x:v>257</x:v>
       </x:c>
-      <x:c r="C39" s="1" t="s">
+      <x:c r="D39" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E39" s="1" t="s">
         <x:v>258</x:v>
-      </x:c>
-      <x:c r="D39" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E39" s="1" t="s">
-        <x:v>259</x:v>
       </x:c>
       <x:c r="L39" s="1" t="s">
         <x:v>42</x:v>
@@ -5315,16 +5312,16 @@
     </x:row>
     <x:row r="40" s="1" customFormat="1">
       <x:c r="B40" s="1" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="C40" s="1" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="C40" s="1" t="s">
+      <x:c r="D40" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E40" s="1" t="s">
         <x:v>261</x:v>
-      </x:c>
-      <x:c r="D40" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E40" s="1" t="s">
-        <x:v>262</x:v>
       </x:c>
       <x:c r="L40" s="1" t="s">
         <x:v>46</x:v>
@@ -5338,16 +5335,16 @@
     </x:row>
     <x:row r="41" s="1" customFormat="1">
       <x:c r="B41" s="1" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="C41" s="1" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="C41" s="1" t="s">
+      <x:c r="D41" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E41" s="1" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="D41" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E41" s="1" t="s">
-        <x:v>265</x:v>
       </x:c>
       <x:c r="L41" s="1" t="s">
         <x:v>50</x:v>
@@ -5355,30 +5352,30 @@
     </x:row>
     <x:row r="42" s="1" customFormat="1">
       <x:c r="B42" s="1" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="C42" s="1" t="s">
         <x:v>266</x:v>
       </x:c>
-      <x:c r="C42" s="1" t="s">
+      <x:c r="D42" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E42" s="1" t="s">
         <x:v>267</x:v>
-      </x:c>
-      <x:c r="D42" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E42" s="1" t="s">
-        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="43" s="1" customFormat="1">
       <x:c r="B43" s="1" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="C43" s="1" t="s">
         <x:v>269</x:v>
       </x:c>
-      <x:c r="C43" s="1" t="s">
+      <x:c r="D43" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E43" s="1" t="s">
         <x:v>270</x:v>
-      </x:c>
-      <x:c r="D43" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E43" s="1" t="s">
-        <x:v>271</x:v>
       </x:c>
       <x:c r="L43" s="1" t="s">
         <x:v>54</x:v>
@@ -5386,16 +5383,16 @@
     </x:row>
     <x:row r="44" s="1" customFormat="1">
       <x:c r="B44" s="1" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="C44" s="1" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="C44" s="1" t="s">
+      <x:c r="D44" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E44" s="1" t="s">
         <x:v>273</x:v>
-      </x:c>
-      <x:c r="D44" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E44" s="1" t="s">
-        <x:v>274</x:v>
       </x:c>
       <x:c r="L44" s="1" t="s">
         <x:v>58</x:v>
@@ -5403,16 +5400,16 @@
     </x:row>
     <x:row r="45" s="1" customFormat="1">
       <x:c r="B45" s="1" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="C45" s="1" t="s">
         <x:v>275</x:v>
       </x:c>
-      <x:c r="C45" s="1" t="s">
+      <x:c r="D45" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E45" s="1" t="s">
         <x:v>276</x:v>
-      </x:c>
-      <x:c r="D45" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E45" s="1" t="s">
-        <x:v>277</x:v>
       </x:c>
       <x:c r="L45" s="1" t="s">
         <x:v>61</x:v>
@@ -5420,16 +5417,16 @@
     </x:row>
     <x:row r="46" s="1" customFormat="1">
       <x:c r="B46" s="1" t="s">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="C46" s="1" t="s">
         <x:v>278</x:v>
       </x:c>
-      <x:c r="C46" s="1" t="s">
+      <x:c r="D46" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E46" s="1" t="s">
         <x:v>279</x:v>
-      </x:c>
-      <x:c r="D46" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E46" s="1" t="s">
-        <x:v>280</x:v>
       </x:c>
       <x:c r="L46" s="1" t="s">
         <x:v>64</x:v>
@@ -5437,16 +5434,16 @@
     </x:row>
     <x:row r="47" s="1" customFormat="1">
       <x:c r="B47" s="1" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="C47" s="1" t="s">
         <x:v>281</x:v>
       </x:c>
-      <x:c r="C47" s="1" t="s">
+      <x:c r="D47" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E47" s="1" t="s">
         <x:v>282</x:v>
-      </x:c>
-      <x:c r="D47" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E47" s="1" t="s">
-        <x:v>283</x:v>
       </x:c>
       <x:c r="L47" s="1" t="s">
         <x:v>67</x:v>
@@ -5454,16 +5451,16 @@
     </x:row>
     <x:row r="48" s="1" customFormat="1">
       <x:c r="B48" s="1" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="C48" s="1" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="C48" s="1" t="s">
+      <x:c r="D48" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E48" s="1" t="s">
         <x:v>285</x:v>
-      </x:c>
-      <x:c r="D48" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E48" s="1" t="s">
-        <x:v>286</x:v>
       </x:c>
       <x:c r="L48" s="1" t="s">
         <x:v>70</x:v>
@@ -5471,16 +5468,16 @@
     </x:row>
     <x:row r="49" s="1" customFormat="1">
       <x:c r="B49" s="1" t="s">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="C49" s="1" t="s">
         <x:v>287</x:v>
       </x:c>
-      <x:c r="C49" s="1" t="s">
+      <x:c r="D49" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E49" s="1" t="s">
         <x:v>288</x:v>
-      </x:c>
-      <x:c r="D49" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E49" s="1" t="s">
-        <x:v>289</x:v>
       </x:c>
       <x:c r="L49" s="1" t="s">
         <x:v>73</x:v>
@@ -5488,414 +5485,414 @@
     </x:row>
     <x:row r="50" s="1" customFormat="1">
       <x:c r="B50" s="1" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="C50" s="1" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="C50" s="1" t="s">
+      <x:c r="D50" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E50" s="1" t="s">
         <x:v>291</x:v>
-      </x:c>
-      <x:c r="D50" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E50" s="1" t="s">
-        <x:v>292</x:v>
       </x:c>
     </x:row>
     <x:row r="51" s="1" customFormat="1">
       <x:c r="B51" s="1" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="C51" s="1" t="s">
         <x:v>293</x:v>
       </x:c>
-      <x:c r="C51" s="1" t="s">
+      <x:c r="D51" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E51" s="1" t="s">
         <x:v>294</x:v>
-      </x:c>
-      <x:c r="D51" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E51" s="1" t="s">
-        <x:v>295</x:v>
       </x:c>
     </x:row>
     <x:row r="52" s="1" customFormat="1">
       <x:c r="B52" s="1" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="C52" s="1" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="C52" s="1" t="s">
+      <x:c r="D52" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E52" s="1" t="s">
         <x:v>297</x:v>
-      </x:c>
-      <x:c r="D52" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E52" s="1" t="s">
-        <x:v>298</x:v>
       </x:c>
     </x:row>
     <x:row r="53" s="1" customFormat="1">
       <x:c r="B53" s="1" t="s">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="C53" s="1" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="C53" s="1" t="s">
+      <x:c r="D53" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E53" s="1" t="s">
         <x:v>300</x:v>
-      </x:c>
-      <x:c r="D53" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E53" s="1" t="s">
-        <x:v>301</x:v>
       </x:c>
     </x:row>
     <x:row r="54" s="1" customFormat="1">
       <x:c r="B54" s="1" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="C54" s="1" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="C54" s="1" t="s">
+      <x:c r="D54" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E54" s="1" t="s">
         <x:v>303</x:v>
-      </x:c>
-      <x:c r="D54" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E54" s="1" t="s">
-        <x:v>304</x:v>
       </x:c>
     </x:row>
     <x:row r="55" s="1" customFormat="1">
       <x:c r="B55" s="1" t="s">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="C55" s="1" t="s">
         <x:v>305</x:v>
       </x:c>
-      <x:c r="C55" s="1" t="s">
+      <x:c r="D55" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E55" s="1" t="s">
         <x:v>306</x:v>
-      </x:c>
-      <x:c r="D55" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E55" s="1" t="s">
-        <x:v>307</x:v>
       </x:c>
     </x:row>
     <x:row r="56" s="1" customFormat="1">
       <x:c r="B56" s="1" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="C56" s="1" t="s">
         <x:v>308</x:v>
       </x:c>
-      <x:c r="C56" s="1" t="s">
+      <x:c r="D56" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E56" s="1" t="s">
         <x:v>309</x:v>
-      </x:c>
-      <x:c r="D56" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E56" s="1" t="s">
-        <x:v>310</x:v>
       </x:c>
     </x:row>
     <x:row r="57" s="1" customFormat="1">
       <x:c r="B57" s="1" t="s">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="C57" s="1" t="s">
         <x:v>311</x:v>
       </x:c>
-      <x:c r="C57" s="1" t="s">
+      <x:c r="D57" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E57" s="1" t="s">
         <x:v>312</x:v>
-      </x:c>
-      <x:c r="D57" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E57" s="1" t="s">
-        <x:v>313</x:v>
       </x:c>
     </x:row>
     <x:row r="58" s="1" customFormat="1">
       <x:c r="B58" s="1" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="C58" s="1" t="s">
         <x:v>314</x:v>
       </x:c>
-      <x:c r="C58" s="1" t="s">
+      <x:c r="D58" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E58" s="1" t="s">
         <x:v>315</x:v>
-      </x:c>
-      <x:c r="D58" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E58" s="1" t="s">
-        <x:v>316</x:v>
       </x:c>
     </x:row>
     <x:row r="59" s="1" customFormat="1">
       <x:c r="B59" s="1" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="C59" s="1" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="C59" s="1" t="s">
+      <x:c r="D59" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E59" s="1" t="s">
         <x:v>318</x:v>
-      </x:c>
-      <x:c r="D59" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E59" s="1" t="s">
-        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="60" s="1" customFormat="1">
       <x:c r="B60" s="1" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="C60" s="1" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="C60" s="1" t="s">
+      <x:c r="D60" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E60" s="1" t="s">
         <x:v>321</x:v>
-      </x:c>
-      <x:c r="D60" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E60" s="1" t="s">
-        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="61" s="1" customFormat="1">
       <x:c r="B61" s="1" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C61" s="1" t="s">
         <x:v>323</x:v>
       </x:c>
-      <x:c r="C61" s="1" t="s">
+      <x:c r="D61" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E61" s="1" t="s">
         <x:v>324</x:v>
-      </x:c>
-      <x:c r="D61" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E61" s="1" t="s">
-        <x:v>325</x:v>
       </x:c>
     </x:row>
     <x:row r="62" s="1" customFormat="1">
       <x:c r="B62" s="1" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="C62" s="1" t="s">
         <x:v>326</x:v>
       </x:c>
-      <x:c r="C62" s="1" t="s">
+      <x:c r="D62" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E62" s="1" t="s">
         <x:v>327</x:v>
-      </x:c>
-      <x:c r="D62" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E62" s="1" t="s">
-        <x:v>328</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="1" customFormat="1">
       <x:c r="B63" s="1" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="C63" s="1" t="s">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="C63" s="1" t="s">
+      <x:c r="D63" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E63" s="1" t="s">
         <x:v>330</x:v>
-      </x:c>
-      <x:c r="D63" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E63" s="1" t="s">
-        <x:v>331</x:v>
       </x:c>
     </x:row>
     <x:row r="64" s="1" customFormat="1">
       <x:c r="B64" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="C64" s="1" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="C64" s="1" t="s">
+      <x:c r="D64" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E64" s="1" t="s">
         <x:v>333</x:v>
-      </x:c>
-      <x:c r="D64" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E64" s="1" t="s">
-        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="65" s="1" customFormat="1">
       <x:c r="B65" s="1" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="C65" s="1" t="s">
         <x:v>335</x:v>
       </x:c>
-      <x:c r="C65" s="1" t="s">
+      <x:c r="D65" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E65" s="1" t="s">
         <x:v>336</x:v>
-      </x:c>
-      <x:c r="D65" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E65" s="1" t="s">
-        <x:v>337</x:v>
       </x:c>
     </x:row>
     <x:row r="66" s="1" customFormat="1">
       <x:c r="B66" s="1" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="C66" s="1" t="s">
         <x:v>338</x:v>
       </x:c>
-      <x:c r="C66" s="1" t="s">
+      <x:c r="D66" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E66" s="1" t="s">
         <x:v>339</x:v>
-      </x:c>
-      <x:c r="D66" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E66" s="1" t="s">
-        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="67" s="1" customFormat="1">
       <x:c r="B67" s="1" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="C67" s="1" t="s">
         <x:v>341</x:v>
       </x:c>
-      <x:c r="C67" s="1" t="s">
+      <x:c r="D67" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E67" s="1" t="s">
         <x:v>342</x:v>
-      </x:c>
-      <x:c r="D67" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E67" s="1" t="s">
-        <x:v>343</x:v>
       </x:c>
     </x:row>
     <x:row r="68" s="1" customFormat="1">
       <x:c r="B68" s="1" t="s">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="C68" s="1" t="s">
         <x:v>344</x:v>
       </x:c>
-      <x:c r="C68" s="1" t="s">
+      <x:c r="D68" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E68" s="1" t="s">
         <x:v>345</x:v>
-      </x:c>
-      <x:c r="D68" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E68" s="1" t="s">
-        <x:v>346</x:v>
       </x:c>
     </x:row>
     <x:row r="69" s="1" customFormat="1">
       <x:c r="B69" s="1" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="C69" s="1" t="s">
         <x:v>347</x:v>
       </x:c>
-      <x:c r="C69" s="1" t="s">
+      <x:c r="D69" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E69" s="1" t="s">
         <x:v>348</x:v>
-      </x:c>
-      <x:c r="D69" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E69" s="1" t="s">
-        <x:v>349</x:v>
       </x:c>
     </x:row>
     <x:row r="70" s="1" customFormat="1">
       <x:c r="B70" s="1" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="C70" s="1" t="s">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="C70" s="1" t="s">
+      <x:c r="D70" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E70" s="1" t="s">
         <x:v>351</x:v>
-      </x:c>
-      <x:c r="D70" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E70" s="1" t="s">
-        <x:v>352</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="1" customFormat="1">
       <x:c r="B71" s="1" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="C71" s="1" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="C71" s="1" t="s">
+      <x:c r="D71" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E71" s="1" t="s">
         <x:v>354</x:v>
-      </x:c>
-      <x:c r="D71" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E71" s="1" t="s">
-        <x:v>355</x:v>
       </x:c>
     </x:row>
     <x:row r="72" s="1" customFormat="1">
       <x:c r="B72" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="C72" s="1" t="s">
         <x:v>356</x:v>
       </x:c>
-      <x:c r="C72" s="1" t="s">
+      <x:c r="D72" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E72" s="1" t="s">
         <x:v>357</x:v>
-      </x:c>
-      <x:c r="D72" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E72" s="1" t="s">
-        <x:v>358</x:v>
       </x:c>
     </x:row>
     <x:row r="73" s="1" customFormat="1">
       <x:c r="B73" s="1" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="C73" s="1" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="C73" s="1" t="s">
+      <x:c r="D73" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E73" s="1" t="s">
         <x:v>360</x:v>
-      </x:c>
-      <x:c r="D73" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E73" s="1" t="s">
-        <x:v>361</x:v>
       </x:c>
     </x:row>
     <x:row r="74" s="1" customFormat="1">
       <x:c r="B74" s="1" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="C74" s="1" t="s">
         <x:v>362</x:v>
       </x:c>
-      <x:c r="C74" s="1" t="s">
+      <x:c r="D74" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E74" s="1" t="s">
         <x:v>363</x:v>
-      </x:c>
-      <x:c r="D74" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E74" s="1" t="s">
-        <x:v>364</x:v>
       </x:c>
     </x:row>
     <x:row r="75" s="1" customFormat="1">
       <x:c r="B75" s="1" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="C75" s="1" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="C75" s="1" t="s">
+      <x:c r="D75" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E75" s="1" t="s">
         <x:v>366</x:v>
-      </x:c>
-      <x:c r="D75" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E75" s="1" t="s">
-        <x:v>367</x:v>
       </x:c>
     </x:row>
     <x:row r="76" s="1" customFormat="1">
       <x:c r="B76" s="1" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="C76" s="1" t="s">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="C76" s="1" t="s">
+      <x:c r="D76" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E76" s="1" t="s">
         <x:v>369</x:v>
-      </x:c>
-      <x:c r="D76" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E76" s="1" t="s">
-        <x:v>370</x:v>
       </x:c>
     </x:row>
     <x:row r="77" s="1" customFormat="1">
       <x:c r="B77" s="1" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="C77" s="1" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="C77" s="1" t="s">
+      <x:c r="D77" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E77" s="1" t="s">
         <x:v>372</x:v>
-      </x:c>
-      <x:c r="D77" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E77" s="1" t="s">
-        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="78" s="1" customFormat="1">
       <x:c r="B78" s="1" t="s">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="C78" s="1" t="s">
         <x:v>374</x:v>
       </x:c>
-      <x:c r="C78" s="1" t="s">
+      <x:c r="D78" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E78" s="1" t="s">
         <x:v>375</x:v>
       </x:c>
-      <x:c r="D78" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E78" s="1" t="s">
+      <x:c r="Q78" s="1" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="Q78" s="1" t="s">
+      <x:c r="R78" s="1" t="s">
         <x:v>377</x:v>
-      </x:c>
-      <x:c r="R78" s="1" t="s">
-        <x:v>378</x:v>
       </x:c>
       <x:c r="S78" s="1">
         <x:v>80</x:v>
@@ -5906,16 +5903,16 @@
     </x:row>
     <x:row r="79" s="1" customFormat="1">
       <x:c r="B79" s="1" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="C79" s="1" t="s">
         <x:v>379</x:v>
       </x:c>
-      <x:c r="C79" s="1" t="s">
+      <x:c r="D79" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E79" s="1" t="s">
         <x:v>380</x:v>
-      </x:c>
-      <x:c r="D79" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E79" s="1" t="s">
-        <x:v>381</x:v>
       </x:c>
       <x:c r="T79" s="1" t="s">
         <x:v>46</x:v>
@@ -5923,16 +5920,16 @@
     </x:row>
     <x:row r="80" s="1" customFormat="1">
       <x:c r="B80" s="1" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="C80" s="1" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="C80" s="1" t="s">
+      <x:c r="D80" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E80" s="1" t="s">
         <x:v>383</x:v>
-      </x:c>
-      <x:c r="D80" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E80" s="1" t="s">
-        <x:v>384</x:v>
       </x:c>
       <x:c r="T80" s="1" t="s">
         <x:v>50</x:v>
@@ -5940,22 +5937,22 @@
     </x:row>
     <x:row r="81" s="1" customFormat="1">
       <x:c r="B81" s="1" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="C81" s="1" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="C81" s="1" t="s">
+      <x:c r="D81" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E81" s="1" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="D81" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E81" s="1" t="s">
+      <x:c r="Q81" s="1" t="s">
         <x:v>387</x:v>
       </x:c>
-      <x:c r="Q81" s="1" t="s">
+      <x:c r="R81" s="1" t="s">
         <x:v>388</x:v>
-      </x:c>
-      <x:c r="R81" s="1" t="s">
-        <x:v>389</x:v>
       </x:c>
       <x:c r="S81" s="1">
         <x:v>100</x:v>
@@ -5966,16 +5963,16 @@
     </x:row>
     <x:row r="82" s="1" customFormat="1">
       <x:c r="B82" s="1" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="C82" s="1" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="C82" s="1" t="s">
+      <x:c r="D82" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E82" s="1" t="s">
         <x:v>391</x:v>
-      </x:c>
-      <x:c r="D82" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E82" s="1" t="s">
-        <x:v>392</x:v>
       </x:c>
       <x:c r="T82" s="1" t="s">
         <x:v>67</x:v>
@@ -5983,16 +5980,16 @@
     </x:row>
     <x:row r="83" s="1" customFormat="1">
       <x:c r="B83" s="1" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="C83" s="1" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="C83" s="1" t="s">
+      <x:c r="D83" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E83" s="1" t="s">
         <x:v>394</x:v>
-      </x:c>
-      <x:c r="D83" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E83" s="1" t="s">
-        <x:v>395</x:v>
       </x:c>
       <x:c r="T83" s="1" t="s">
         <x:v>61</x:v>
@@ -6000,22 +5997,22 @@
     </x:row>
     <x:row r="84" s="1" customFormat="1">
       <x:c r="B84" s="1" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="C84" s="1" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="C84" s="1" t="s">
+      <x:c r="D84" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E84" s="1" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="D84" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E84" s="1" t="s">
+      <x:c r="Q84" s="1" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="Q84" s="1" t="s">
+      <x:c r="R84" s="1" t="s">
         <x:v>399</x:v>
-      </x:c>
-      <x:c r="R84" s="1" t="s">
-        <x:v>400</x:v>
       </x:c>
       <x:c r="S84" s="1">
         <x:v>80</x:v>
@@ -6026,16 +6023,16 @@
     </x:row>
     <x:row r="85" s="1" customFormat="1">
       <x:c r="B85" s="1" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="C85" s="1" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="C85" s="1" t="s">
+      <x:c r="D85" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E85" s="1" t="s">
         <x:v>402</x:v>
-      </x:c>
-      <x:c r="D85" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E85" s="1" t="s">
-        <x:v>403</x:v>
       </x:c>
       <x:c r="T85" s="1" t="s">
         <x:v>64</x:v>
@@ -6043,16 +6040,16 @@
     </x:row>
     <x:row r="86" s="1" customFormat="1">
       <x:c r="B86" s="1" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="C86" s="1" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="C86" s="1" t="s">
+      <x:c r="D86" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E86" s="1" t="s">
         <x:v>405</x:v>
-      </x:c>
-      <x:c r="D86" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E86" s="1" t="s">
-        <x:v>406</x:v>
       </x:c>
       <x:c r="T86" s="1" t="s">
         <x:v>67</x:v>
@@ -6060,22 +6057,22 @@
     </x:row>
     <x:row r="87" s="1" customFormat="1">
       <x:c r="B87" s="1" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="C87" s="1" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="C87" s="1" t="s">
+      <x:c r="D87" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E87" s="1" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="D87" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E87" s="1" t="s">
+      <x:c r="Q87" s="1" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="Q87" s="1" t="s">
+      <x:c r="R87" s="1" t="s">
         <x:v>410</x:v>
-      </x:c>
-      <x:c r="R87" s="1" t="s">
-        <x:v>411</x:v>
       </x:c>
       <x:c r="S87" s="1">
         <x:v>100</x:v>
@@ -6086,16 +6083,16 @@
     </x:row>
     <x:row r="88" s="1" customFormat="1">
       <x:c r="B88" s="1" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="C88" s="1" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="C88" s="1" t="s">
+      <x:c r="D88" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E88" s="1" t="s">
         <x:v>413</x:v>
-      </x:c>
-      <x:c r="D88" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E88" s="1" t="s">
-        <x:v>414</x:v>
       </x:c>
       <x:c r="T88" s="1" t="s">
         <x:v>31</x:v>
@@ -6103,16 +6100,16 @@
     </x:row>
     <x:row r="89" s="1" customFormat="1">
       <x:c r="B89" s="1" t="s">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="C89" s="1" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="C89" s="1" t="s">
+      <x:c r="D89" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E89" s="1" t="s">
         <x:v>416</x:v>
-      </x:c>
-      <x:c r="D89" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E89" s="1" t="s">
-        <x:v>417</x:v>
       </x:c>
       <x:c r="T89" s="1" t="s">
         <x:v>50</x:v>
@@ -6120,22 +6117,22 @@
     </x:row>
     <x:row r="90" s="1" customFormat="1">
       <x:c r="B90" s="1" t="s">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="C90" s="1" t="s">
         <x:v>418</x:v>
       </x:c>
-      <x:c r="C90" s="1" t="s">
+      <x:c r="D90" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E90" s="1" t="s">
         <x:v>419</x:v>
       </x:c>
-      <x:c r="D90" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E90" s="1" t="s">
+      <x:c r="Q90" s="1" t="s">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="Q90" s="1" t="s">
+      <x:c r="R90" s="1" t="s">
         <x:v>421</x:v>
-      </x:c>
-      <x:c r="R90" s="1" t="s">
-        <x:v>422</x:v>
       </x:c>
       <x:c r="S90" s="1">
         <x:v>100</x:v>
@@ -6146,16 +6143,16 @@
     </x:row>
     <x:row r="91" s="1" customFormat="1">
       <x:c r="B91" s="1" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="C91" s="1" t="s">
         <x:v>423</x:v>
       </x:c>
-      <x:c r="C91" s="1" t="s">
+      <x:c r="D91" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E91" s="1" t="s">
         <x:v>424</x:v>
-      </x:c>
-      <x:c r="D91" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E91" s="1" t="s">
-        <x:v>425</x:v>
       </x:c>
       <x:c r="T91" s="1" t="s">
         <x:v>77</x:v>
@@ -6163,22 +6160,22 @@
     </x:row>
     <x:row r="92" s="1" customFormat="1">
       <x:c r="B92" s="1" t="s">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="C92" s="1" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="C92" s="1" t="s">
+      <x:c r="D92" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E92" s="1" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="D92" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E92" s="1" t="s">
+      <x:c r="Q92" s="1" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="Q92" s="1" t="s">
+      <x:c r="R92" s="1" t="s">
         <x:v>429</x:v>
-      </x:c>
-      <x:c r="R92" s="1" t="s">
-        <x:v>430</x:v>
       </x:c>
       <x:c r="S92" s="1">
         <x:v>100</x:v>
@@ -6189,444 +6186,444 @@
     </x:row>
     <x:row r="93" s="1" customFormat="1">
       <x:c r="B93" s="1" t="s">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="C93" s="1" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="C93" s="1" t="s">
+      <x:c r="D93" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E93" s="1" t="s">
         <x:v>432</x:v>
-      </x:c>
-      <x:c r="D93" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E93" s="1" t="s">
-        <x:v>433</x:v>
       </x:c>
     </x:row>
     <x:row r="94" s="1" customFormat="1">
       <x:c r="B94" s="1" t="s">
+        <x:v>433</x:v>
+      </x:c>
+      <x:c r="C94" s="1" t="s">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="C94" s="1" t="s">
+      <x:c r="D94" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E94" s="1" t="s">
         <x:v>435</x:v>
-      </x:c>
-      <x:c r="D94" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E94" s="1" t="s">
-        <x:v>436</x:v>
       </x:c>
     </x:row>
     <x:row r="95" s="1" customFormat="1">
       <x:c r="B95" s="1" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="C95" s="1" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="C95" s="1" t="s">
+      <x:c r="D95" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E95" s="1" t="s">
         <x:v>438</x:v>
-      </x:c>
-      <x:c r="D95" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E95" s="1" t="s">
-        <x:v>439</x:v>
       </x:c>
     </x:row>
     <x:row r="96" s="1" customFormat="1">
       <x:c r="B96" s="1" t="s">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="C96" s="1" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="C96" s="1" t="s">
+      <x:c r="D96" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E96" s="1" t="s">
         <x:v>441</x:v>
-      </x:c>
-      <x:c r="D96" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E96" s="1" t="s">
-        <x:v>442</x:v>
       </x:c>
     </x:row>
     <x:row r="97" s="1" customFormat="1">
       <x:c r="B97" s="1" t="s">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="C97" s="1" t="s">
         <x:v>443</x:v>
       </x:c>
-      <x:c r="C97" s="1" t="s">
+      <x:c r="D97" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E97" s="1" t="s">
         <x:v>444</x:v>
-      </x:c>
-      <x:c r="D97" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E97" s="1" t="s">
-        <x:v>445</x:v>
       </x:c>
     </x:row>
     <x:row r="98" s="1" customFormat="1">
       <x:c r="B98" s="1" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="C98" s="1" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="C98" s="1" t="s">
+      <x:c r="D98" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E98" s="1" t="s">
         <x:v>447</x:v>
-      </x:c>
-      <x:c r="D98" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E98" s="1" t="s">
-        <x:v>448</x:v>
       </x:c>
     </x:row>
     <x:row r="99" s="1" customFormat="1">
       <x:c r="B99" s="1" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="C99" s="1" t="s">
         <x:v>449</x:v>
       </x:c>
-      <x:c r="C99" s="1" t="s">
+      <x:c r="D99" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E99" s="1" t="s">
         <x:v>450</x:v>
-      </x:c>
-      <x:c r="D99" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E99" s="1" t="s">
-        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="100" s="1" customFormat="1">
       <x:c r="B100" s="1" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C100" s="1" t="s">
         <x:v>452</x:v>
       </x:c>
-      <x:c r="C100" s="1" t="s">
+      <x:c r="D100" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E100" s="1" t="s">
         <x:v>453</x:v>
-      </x:c>
-      <x:c r="D100" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E100" s="1" t="s">
-        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="101" s="1" customFormat="1">
       <x:c r="B101" s="1" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="C101" s="1" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="C101" s="1" t="s">
+      <x:c r="D101" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E101" s="1" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="D101" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E101" s="1" t="s">
-        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="102" s="1" customFormat="1">
       <x:c r="B102" s="1" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="C102" s="1" t="s">
         <x:v>458</x:v>
       </x:c>
-      <x:c r="C102" s="1" t="s">
+      <x:c r="D102" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E102" s="1" t="s">
         <x:v>459</x:v>
-      </x:c>
-      <x:c r="D102" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E102" s="1" t="s">
-        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="103" s="1" customFormat="1">
       <x:c r="B103" s="1" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="C103" s="1" t="s">
         <x:v>461</x:v>
       </x:c>
-      <x:c r="C103" s="1" t="s">
+      <x:c r="D103" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E103" s="1" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="D103" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E103" s="1" t="s">
-        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="104" s="1" customFormat="1">
       <x:c r="B104" s="1" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="C104" s="1" t="s">
         <x:v>464</x:v>
       </x:c>
-      <x:c r="C104" s="1" t="s">
+      <x:c r="D104" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E104" s="1" t="s">
         <x:v>465</x:v>
-      </x:c>
-      <x:c r="D104" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E104" s="1" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="105" s="1" customFormat="1">
       <x:c r="B105" s="1" t="s">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="C105" s="1" t="s">
         <x:v>467</x:v>
       </x:c>
-      <x:c r="C105" s="1" t="s">
+      <x:c r="D105" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E105" s="1" t="s">
         <x:v>468</x:v>
-      </x:c>
-      <x:c r="D105" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E105" s="1" t="s">
-        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="106" s="1" customFormat="1">
       <x:c r="B106" s="1" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C106" s="1" t="s">
         <x:v>470</x:v>
       </x:c>
-      <x:c r="C106" s="1" t="s">
+      <x:c r="D106" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E106" s="1" t="s">
         <x:v>471</x:v>
-      </x:c>
-      <x:c r="D106" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E106" s="1" t="s">
-        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="107" s="1" customFormat="1">
       <x:c r="B107" s="1" t="s">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="C107" s="1" t="s">
         <x:v>473</x:v>
       </x:c>
-      <x:c r="C107" s="1" t="s">
+      <x:c r="D107" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E107" s="1" t="s">
         <x:v>474</x:v>
-      </x:c>
-      <x:c r="D107" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E107" s="1" t="s">
-        <x:v>475</x:v>
       </x:c>
     </x:row>
     <x:row r="108" s="1" customFormat="1">
       <x:c r="B108" s="1" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="C108" s="1" t="s">
         <x:v>476</x:v>
       </x:c>
-      <x:c r="C108" s="1" t="s">
+      <x:c r="D108" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E108" s="1" t="s">
         <x:v>477</x:v>
-      </x:c>
-      <x:c r="D108" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E108" s="1" t="s">
-        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="109" s="1" customFormat="1">
       <x:c r="B109" s="1" t="s">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="C109" s="1" t="s">
         <x:v>479</x:v>
       </x:c>
-      <x:c r="C109" s="1" t="s">
+      <x:c r="D109" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E109" s="1" t="s">
         <x:v>480</x:v>
-      </x:c>
-      <x:c r="D109" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E109" s="1" t="s">
-        <x:v>481</x:v>
       </x:c>
     </x:row>
     <x:row r="110" s="1" customFormat="1">
       <x:c r="B110" s="1" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="C110" s="1" t="s">
         <x:v>482</x:v>
       </x:c>
-      <x:c r="C110" s="1" t="s">
+      <x:c r="D110" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E110" s="1" t="s">
         <x:v>483</x:v>
-      </x:c>
-      <x:c r="D110" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E110" s="1" t="s">
-        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="111" s="1" customFormat="1">
       <x:c r="B111" s="1" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="C111" s="1" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="C111" s="1" t="s">
+      <x:c r="D111" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E111" s="1" t="s">
         <x:v>486</x:v>
-      </x:c>
-      <x:c r="D111" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E111" s="1" t="s">
-        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="112" s="1" customFormat="1">
       <x:c r="B112" s="1" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="C112" s="1" t="s">
         <x:v>488</x:v>
       </x:c>
-      <x:c r="C112" s="1" t="s">
+      <x:c r="D112" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E112" s="1" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="D112" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E112" s="1" t="s">
-        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="113" s="1" customFormat="1">
       <x:c r="B113" s="1" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="C113" s="1" t="s">
         <x:v>491</x:v>
       </x:c>
-      <x:c r="C113" s="1" t="s">
+      <x:c r="D113" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E113" s="1" t="s">
         <x:v>492</x:v>
-      </x:c>
-      <x:c r="D113" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E113" s="1" t="s">
-        <x:v>493</x:v>
       </x:c>
     </x:row>
     <x:row r="114" s="1" customFormat="1">
       <x:c r="B114" s="1" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="C114" s="1" t="s">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="C114" s="1" t="s">
+      <x:c r="D114" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E114" s="1" t="s">
         <x:v>495</x:v>
-      </x:c>
-      <x:c r="D114" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E114" s="1" t="s">
-        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="115" s="1" customFormat="1">
       <x:c r="B115" s="1" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="C115" s="1" t="s">
         <x:v>497</x:v>
       </x:c>
-      <x:c r="C115" s="1" t="s">
+      <x:c r="D115" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E115" s="1" t="s">
         <x:v>498</x:v>
-      </x:c>
-      <x:c r="D115" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E115" s="1" t="s">
-        <x:v>499</x:v>
       </x:c>
     </x:row>
     <x:row r="116" s="1" customFormat="1">
       <x:c r="B116" s="1" t="s">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="C116" s="1" t="s">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="C116" s="1" t="s">
+      <x:c r="D116" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E116" s="1" t="s">
         <x:v>501</x:v>
-      </x:c>
-      <x:c r="D116" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E116" s="1" t="s">
-        <x:v>502</x:v>
       </x:c>
     </x:row>
     <x:row r="117" s="1" customFormat="1">
       <x:c r="B117" s="1" t="s">
+        <x:v>502</x:v>
+      </x:c>
+      <x:c r="C117" s="1" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="C117" s="1" t="s">
+      <x:c r="D117" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E117" s="1" t="s">
         <x:v>504</x:v>
-      </x:c>
-      <x:c r="D117" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E117" s="1" t="s">
-        <x:v>505</x:v>
       </x:c>
     </x:row>
     <x:row r="118" s="1" customFormat="1">
       <x:c r="B118" s="1" t="s">
+        <x:v>505</x:v>
+      </x:c>
+      <x:c r="C118" s="1" t="s">
         <x:v>506</x:v>
       </x:c>
-      <x:c r="C118" s="1" t="s">
+      <x:c r="D118" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E118" s="1" t="s">
         <x:v>507</x:v>
-      </x:c>
-      <x:c r="D118" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E118" s="1" t="s">
-        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="119" s="1" customFormat="1">
       <x:c r="B119" s="1" t="s">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="C119" s="1" t="s">
         <x:v>509</x:v>
       </x:c>
-      <x:c r="C119" s="1" t="s">
+      <x:c r="D119" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E119" s="1" t="s">
         <x:v>510</x:v>
-      </x:c>
-      <x:c r="D119" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E119" s="1" t="s">
-        <x:v>511</x:v>
       </x:c>
     </x:row>
     <x:row r="120" s="1" customFormat="1">
       <x:c r="B120" s="1" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="C120" s="1" t="s">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="C120" s="1" t="s">
+      <x:c r="D120" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E120" s="1" t="s">
         <x:v>513</x:v>
-      </x:c>
-      <x:c r="D120" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E120" s="1" t="s">
-        <x:v>514</x:v>
       </x:c>
     </x:row>
     <x:row r="121" s="1" customFormat="1">
       <x:c r="B121" s="1" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="C121" s="1" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="C121" s="1" t="s">
+      <x:c r="D121" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E121" s="1" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="D121" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E121" s="1" t="s">
-        <x:v>517</x:v>
       </x:c>
     </x:row>
     <x:row r="122" s="1" customFormat="1">
       <x:c r="B122" s="1" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="C122" s="1" t="s">
         <x:v>518</x:v>
       </x:c>
-      <x:c r="C122" s="1" t="s">
+      <x:c r="D122" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E122" s="1" t="s">
         <x:v>519</x:v>
-      </x:c>
-      <x:c r="D122" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E122" s="1" t="s">
-        <x:v>520</x:v>
       </x:c>
     </x:row>
     <x:row r="123" s="1" customFormat="1">
       <x:c r="B123" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="C123" s="1" t="s">
         <x:v>521</x:v>
       </x:c>
-      <x:c r="C123" s="1" t="s">
+      <x:c r="D123" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E123" s="1" t="s">
         <x:v>522</x:v>
-      </x:c>
-      <x:c r="D123" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E123" s="1" t="s">
-        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="124" s="1" customFormat="1">
       <x:c r="B124" s="1" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C124" s="1" t="s">
-        <x:v>524</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="D124" s="1">
         <x:v>100</x:v>
@@ -6637,10 +6634,10 @@
     </x:row>
     <x:row r="125" s="1" customFormat="1">
       <x:c r="B125" s="1" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="C125" s="1" t="s">
         <x:v>525</x:v>
-      </x:c>
-      <x:c r="C125" s="1" t="s">
-        <x:v>526</x:v>
       </x:c>
       <x:c r="D125" s="1">
         <x:v>100</x:v>
@@ -6651,570 +6648,570 @@
     </x:row>
     <x:row r="126" s="1" customFormat="1">
       <x:c r="B126" s="1" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="C126" s="1" t="s">
         <x:v>527</x:v>
       </x:c>
-      <x:c r="C126" s="1" t="s">
+      <x:c r="D126" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E126" s="1" t="s">
         <x:v>528</x:v>
-      </x:c>
-      <x:c r="D126" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E126" s="1" t="s">
-        <x:v>529</x:v>
       </x:c>
     </x:row>
     <x:row r="127" s="1" customFormat="1">
       <x:c r="B127" s="1" t="s">
+        <x:v>529</x:v>
+      </x:c>
+      <x:c r="C127" s="1" t="s">
         <x:v>530</x:v>
       </x:c>
-      <x:c r="C127" s="1" t="s">
+      <x:c r="D127" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E127" s="1" t="s">
         <x:v>531</x:v>
-      </x:c>
-      <x:c r="D127" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E127" s="1" t="s">
-        <x:v>532</x:v>
       </x:c>
     </x:row>
     <x:row r="128" s="1" customFormat="1">
       <x:c r="B128" s="1" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="C128" s="1" t="s">
         <x:v>533</x:v>
       </x:c>
-      <x:c r="C128" s="1" t="s">
+      <x:c r="D128" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E128" s="1" t="s">
         <x:v>534</x:v>
-      </x:c>
-      <x:c r="D128" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E128" s="1" t="s">
-        <x:v>535</x:v>
       </x:c>
     </x:row>
     <x:row r="129" s="1" customFormat="1">
       <x:c r="B129" s="1" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="C129" s="1" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="C129" s="1" t="s">
+      <x:c r="D129" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E129" s="1" t="s">
         <x:v>537</x:v>
-      </x:c>
-      <x:c r="D129" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E129" s="1" t="s">
-        <x:v>538</x:v>
       </x:c>
     </x:row>
     <x:row r="130" s="1" customFormat="1">
       <x:c r="B130" s="1" t="s">
+        <x:v>538</x:v>
+      </x:c>
+      <x:c r="C130" s="1" t="s">
         <x:v>539</x:v>
       </x:c>
-      <x:c r="C130" s="1" t="s">
+      <x:c r="D130" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E130" s="1" t="s">
         <x:v>540</x:v>
-      </x:c>
-      <x:c r="D130" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E130" s="1" t="s">
-        <x:v>541</x:v>
       </x:c>
     </x:row>
     <x:row r="131" s="1" customFormat="1">
       <x:c r="B131" s="1" t="s">
+        <x:v>541</x:v>
+      </x:c>
+      <x:c r="C131" s="1" t="s">
         <x:v>542</x:v>
       </x:c>
-      <x:c r="C131" s="1" t="s">
+      <x:c r="D131" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E131" s="1" t="s">
         <x:v>543</x:v>
-      </x:c>
-      <x:c r="D131" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E131" s="1" t="s">
-        <x:v>544</x:v>
       </x:c>
     </x:row>
     <x:row r="132" s="1" customFormat="1">
       <x:c r="B132" s="1" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="C132" s="1" t="s">
         <x:v>545</x:v>
       </x:c>
-      <x:c r="C132" s="1" t="s">
+      <x:c r="D132" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E132" s="1" t="s">
         <x:v>546</x:v>
-      </x:c>
-      <x:c r="D132" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E132" s="1" t="s">
-        <x:v>547</x:v>
       </x:c>
     </x:row>
     <x:row r="133" s="1" customFormat="1">
       <x:c r="B133" s="1" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="C133" s="1" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="C133" s="1" t="s">
+      <x:c r="D133" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E133" s="1" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="D133" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E133" s="1" t="s">
-        <x:v>550</x:v>
       </x:c>
     </x:row>
     <x:row r="134" s="1" customFormat="1">
       <x:c r="B134" s="1" t="s">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="C134" s="1" t="s">
         <x:v>551</x:v>
       </x:c>
-      <x:c r="C134" s="1" t="s">
+      <x:c r="D134" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E134" s="1" t="s">
         <x:v>552</x:v>
-      </x:c>
-      <x:c r="D134" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E134" s="1" t="s">
-        <x:v>553</x:v>
       </x:c>
     </x:row>
     <x:row r="135" s="1" customFormat="1">
       <x:c r="B135" s="1" t="s">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="C135" s="1" t="s">
         <x:v>554</x:v>
       </x:c>
-      <x:c r="C135" s="1" t="s">
+      <x:c r="D135" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E135" s="1" t="s">
         <x:v>555</x:v>
-      </x:c>
-      <x:c r="D135" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E135" s="1" t="s">
-        <x:v>556</x:v>
       </x:c>
     </x:row>
     <x:row r="136" s="1" customFormat="1">
       <x:c r="B136" s="1" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="C136" s="1" t="s">
         <x:v>557</x:v>
       </x:c>
-      <x:c r="C136" s="1" t="s">
+      <x:c r="D136" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E136" s="1" t="s">
         <x:v>558</x:v>
-      </x:c>
-      <x:c r="D136" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E136" s="1" t="s">
-        <x:v>559</x:v>
       </x:c>
     </x:row>
     <x:row r="137" s="1" customFormat="1">
       <x:c r="B137" s="1" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="C137" s="1" t="s">
         <x:v>560</x:v>
       </x:c>
-      <x:c r="C137" s="1" t="s">
+      <x:c r="D137" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E137" s="1" t="s">
         <x:v>561</x:v>
-      </x:c>
-      <x:c r="D137" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E137" s="1" t="s">
-        <x:v>562</x:v>
       </x:c>
     </x:row>
     <x:row r="138" s="1" customFormat="1">
       <x:c r="B138" s="1" t="s">
+        <x:v>562</x:v>
+      </x:c>
+      <x:c r="C138" s="1" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="C138" s="1" t="s">
+      <x:c r="D138" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E138" s="1" t="s">
         <x:v>564</x:v>
-      </x:c>
-      <x:c r="D138" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E138" s="1" t="s">
-        <x:v>565</x:v>
       </x:c>
     </x:row>
     <x:row r="139" s="1" customFormat="1">
       <x:c r="B139" s="1" t="s">
+        <x:v>565</x:v>
+      </x:c>
+      <x:c r="C139" s="1" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="C139" s="1" t="s">
+      <x:c r="D139" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E139" s="1" t="s">
         <x:v>567</x:v>
-      </x:c>
-      <x:c r="D139" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E139" s="1" t="s">
-        <x:v>568</x:v>
       </x:c>
     </x:row>
     <x:row r="140" s="1" customFormat="1">
       <x:c r="B140" s="1" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C140" s="1" t="s">
+        <x:v>568</x:v>
+      </x:c>
+      <x:c r="D140" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E140" s="1" t="s">
         <x:v>569</x:v>
-      </x:c>
-      <x:c r="D140" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E140" s="1" t="s">
-        <x:v>570</x:v>
       </x:c>
     </x:row>
     <x:row r="141" s="1" customFormat="1">
       <x:c r="B141" s="1" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C141" s="1" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="D141" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E141" s="1" t="s">
         <x:v>571</x:v>
-      </x:c>
-      <x:c r="D141" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E141" s="1" t="s">
-        <x:v>572</x:v>
       </x:c>
     </x:row>
     <x:row r="142" s="1" customFormat="1">
       <x:c r="B142" s="1" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C142" s="1" t="s">
         <x:v>573</x:v>
       </x:c>
-      <x:c r="C142" s="1" t="s">
+      <x:c r="D142" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E142" s="1" t="s">
         <x:v>574</x:v>
-      </x:c>
-      <x:c r="D142" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E142" s="1" t="s">
-        <x:v>575</x:v>
       </x:c>
     </x:row>
     <x:row r="143" s="1" customFormat="1">
       <x:c r="B143" s="1" t="s">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="C143" s="1" t="s">
         <x:v>576</x:v>
       </x:c>
-      <x:c r="C143" s="1" t="s">
+      <x:c r="D143" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E143" s="1" t="s">
         <x:v>577</x:v>
-      </x:c>
-      <x:c r="D143" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E143" s="1" t="s">
-        <x:v>578</x:v>
       </x:c>
     </x:row>
     <x:row r="144" s="1" customFormat="1">
       <x:c r="B144" s="1" t="s">
+        <x:v>578</x:v>
+      </x:c>
+      <x:c r="C144" s="1" t="s">
         <x:v>579</x:v>
       </x:c>
-      <x:c r="C144" s="1" t="s">
+      <x:c r="D144" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E144" s="1" t="s">
         <x:v>580</x:v>
-      </x:c>
-      <x:c r="D144" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E144" s="1" t="s">
-        <x:v>581</x:v>
       </x:c>
     </x:row>
     <x:row r="145" s="1" customFormat="1">
       <x:c r="B145" s="1" t="s">
+        <x:v>581</x:v>
+      </x:c>
+      <x:c r="C145" s="1" t="s">
         <x:v>582</x:v>
       </x:c>
-      <x:c r="C145" s="1" t="s">
+      <x:c r="D145" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E145" s="1" t="s">
         <x:v>583</x:v>
-      </x:c>
-      <x:c r="D145" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E145" s="1" t="s">
-        <x:v>584</x:v>
       </x:c>
     </x:row>
     <x:row r="146" s="1" customFormat="1">
       <x:c r="B146" s="1" t="s">
+        <x:v>584</x:v>
+      </x:c>
+      <x:c r="C146" s="1" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="C146" s="1" t="s">
+      <x:c r="D146" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E146" s="1" t="s">
         <x:v>586</x:v>
-      </x:c>
-      <x:c r="D146" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E146" s="1" t="s">
-        <x:v>587</x:v>
       </x:c>
     </x:row>
     <x:row r="147" s="1" customFormat="1">
       <x:c r="B147" s="1" t="s">
+        <x:v>587</x:v>
+      </x:c>
+      <x:c r="C147" s="1" t="s">
         <x:v>588</x:v>
       </x:c>
-      <x:c r="C147" s="1" t="s">
+      <x:c r="D147" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E147" s="1" t="s">
         <x:v>589</x:v>
-      </x:c>
-      <x:c r="D147" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E147" s="1" t="s">
-        <x:v>590</x:v>
       </x:c>
     </x:row>
     <x:row r="148" s="1" customFormat="1">
       <x:c r="B148" s="1" t="s">
+        <x:v>590</x:v>
+      </x:c>
+      <x:c r="C148" s="1" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="C148" s="1" t="s">
+      <x:c r="D148" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E148" s="1" t="s">
         <x:v>592</x:v>
-      </x:c>
-      <x:c r="D148" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E148" s="1" t="s">
-        <x:v>593</x:v>
       </x:c>
     </x:row>
     <x:row r="149" s="1" customFormat="1">
       <x:c r="B149" s="1" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="C149" s="1" t="s">
         <x:v>594</x:v>
       </x:c>
-      <x:c r="C149" s="1" t="s">
+      <x:c r="D149" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E149" s="1" t="s">
         <x:v>595</x:v>
-      </x:c>
-      <x:c r="D149" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E149" s="1" t="s">
-        <x:v>596</x:v>
       </x:c>
     </x:row>
     <x:row r="150" s="1" customFormat="1">
       <x:c r="B150" s="1" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="C150" s="1" t="s">
         <x:v>597</x:v>
       </x:c>
-      <x:c r="C150" s="1" t="s">
+      <x:c r="D150" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E150" s="1" t="s">
         <x:v>598</x:v>
-      </x:c>
-      <x:c r="D150" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E150" s="1" t="s">
-        <x:v>599</x:v>
       </x:c>
     </x:row>
     <x:row r="151" s="1" customFormat="1">
       <x:c r="B151" s="1" t="s">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C151" s="1" t="s">
+        <x:v>599</x:v>
+      </x:c>
+      <x:c r="D151" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E151" s="1" t="s">
         <x:v>600</x:v>
-      </x:c>
-      <x:c r="D151" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E151" s="1" t="s">
-        <x:v>601</x:v>
       </x:c>
     </x:row>
     <x:row r="152" s="1" customFormat="1">
       <x:c r="B152" s="1" t="s">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="C152" s="1" t="s">
         <x:v>602</x:v>
       </x:c>
-      <x:c r="C152" s="1" t="s">
+      <x:c r="D152" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E152" s="1" t="s">
         <x:v>603</x:v>
-      </x:c>
-      <x:c r="D152" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E152" s="1" t="s">
-        <x:v>604</x:v>
       </x:c>
     </x:row>
     <x:row r="153" s="1" customFormat="1">
       <x:c r="B153" s="1" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="C153" s="1" t="s">
         <x:v>605</x:v>
       </x:c>
-      <x:c r="C153" s="1" t="s">
+      <x:c r="D153" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E153" s="1" t="s">
         <x:v>606</x:v>
-      </x:c>
-      <x:c r="D153" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E153" s="1" t="s">
-        <x:v>607</x:v>
       </x:c>
     </x:row>
     <x:row r="154" s="1" customFormat="1">
       <x:c r="B154" s="1" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="C154" s="1" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="C154" s="1" t="s">
+      <x:c r="D154" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E154" s="1" t="s">
         <x:v>609</x:v>
-      </x:c>
-      <x:c r="D154" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E154" s="1" t="s">
-        <x:v>610</x:v>
       </x:c>
     </x:row>
     <x:row r="155" s="1" customFormat="1">
       <x:c r="B155" s="1" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="C155" s="1" t="s">
         <x:v>611</x:v>
       </x:c>
-      <x:c r="C155" s="1" t="s">
+      <x:c r="D155" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E155" s="1" t="s">
         <x:v>612</x:v>
-      </x:c>
-      <x:c r="D155" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E155" s="1" t="s">
-        <x:v>613</x:v>
       </x:c>
     </x:row>
     <x:row r="156" s="1" customFormat="1">
       <x:c r="B156" s="1" t="s">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="C156" s="1" t="s">
         <x:v>614</x:v>
       </x:c>
-      <x:c r="C156" s="1" t="s">
+      <x:c r="D156" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E156" s="1" t="s">
         <x:v>615</x:v>
-      </x:c>
-      <x:c r="D156" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E156" s="1" t="s">
-        <x:v>616</x:v>
       </x:c>
     </x:row>
     <x:row r="157" s="1" customFormat="1">
       <x:c r="B157" s="1" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="C157" s="1" t="s">
         <x:v>617</x:v>
       </x:c>
-      <x:c r="C157" s="1" t="s">
+      <x:c r="D157" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E157" s="1" t="s">
         <x:v>618</x:v>
-      </x:c>
-      <x:c r="D157" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E157" s="1" t="s">
-        <x:v>619</x:v>
       </x:c>
     </x:row>
     <x:row r="158" s="1" customFormat="1">
       <x:c r="B158" s="1" t="s">
+        <x:v>619</x:v>
+      </x:c>
+      <x:c r="C158" s="1" t="s">
         <x:v>620</x:v>
       </x:c>
-      <x:c r="C158" s="1" t="s">
+      <x:c r="D158" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E158" s="1" t="s">
         <x:v>621</x:v>
-      </x:c>
-      <x:c r="D158" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E158" s="1" t="s">
-        <x:v>622</x:v>
       </x:c>
     </x:row>
     <x:row r="159" s="1" customFormat="1">
       <x:c r="B159" s="1" t="s">
+        <x:v>622</x:v>
+      </x:c>
+      <x:c r="C159" s="1" t="s">
         <x:v>623</x:v>
       </x:c>
-      <x:c r="C159" s="1" t="s">
+      <x:c r="D159" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E159" s="1" t="s">
         <x:v>624</x:v>
-      </x:c>
-      <x:c r="D159" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E159" s="1" t="s">
-        <x:v>625</x:v>
       </x:c>
     </x:row>
     <x:row r="160" s="1" customFormat="1">
       <x:c r="B160" s="1" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="C160" s="1" t="s">
         <x:v>626</x:v>
       </x:c>
-      <x:c r="C160" s="1" t="s">
+      <x:c r="D160" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E160" s="1" t="s">
         <x:v>627</x:v>
-      </x:c>
-      <x:c r="D160" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E160" s="1" t="s">
-        <x:v>628</x:v>
       </x:c>
     </x:row>
     <x:row r="161" s="1" customFormat="1">
       <x:c r="B161" s="1" t="s">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="C161" s="1" t="s">
         <x:v>629</x:v>
       </x:c>
-      <x:c r="C161" s="1" t="s">
+      <x:c r="D161" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E161" s="1" t="s">
         <x:v>630</x:v>
-      </x:c>
-      <x:c r="D161" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E161" s="1" t="s">
-        <x:v>631</x:v>
       </x:c>
     </x:row>
     <x:row r="162" s="1" customFormat="1">
       <x:c r="B162" s="1" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="C162" s="1" t="s">
         <x:v>632</x:v>
       </x:c>
-      <x:c r="C162" s="1" t="s">
+      <x:c r="D162" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E162" s="1" t="s">
         <x:v>633</x:v>
-      </x:c>
-      <x:c r="D162" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E162" s="1" t="s">
-        <x:v>634</x:v>
       </x:c>
     </x:row>
     <x:row r="163" s="1" customFormat="1">
       <x:c r="B163" s="1" t="s">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="C163" s="1" t="s">
         <x:v>635</x:v>
       </x:c>
-      <x:c r="C163" s="1" t="s">
+      <x:c r="D163" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E163" s="1" t="s">
         <x:v>636</x:v>
-      </x:c>
-      <x:c r="D163" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E163" s="1" t="s">
-        <x:v>637</x:v>
       </x:c>
     </x:row>
     <x:row r="164" s="1" customFormat="1">
       <x:c r="B164" s="1" t="s">
+        <x:v>637</x:v>
+      </x:c>
+      <x:c r="C164" s="1" t="s">
         <x:v>638</x:v>
       </x:c>
-      <x:c r="C164" s="1" t="s">
+      <x:c r="D164" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E164" s="1" t="s">
         <x:v>639</x:v>
-      </x:c>
-      <x:c r="D164" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E164" s="1" t="s">
-        <x:v>640</x:v>
       </x:c>
     </x:row>
     <x:row r="165" s="1" customFormat="1">
       <x:c r="B165" s="1" t="s">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="C165" s="1" t="s">
         <x:v>641</x:v>
       </x:c>
-      <x:c r="C165" s="1" t="s">
+      <x:c r="D165" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E165" s="1" t="s">
         <x:v>642</x:v>
-      </x:c>
-      <x:c r="D165" s="1">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E165" s="1" t="s">
-        <x:v>643</x:v>
       </x:c>
     </x:row>
     <x:row r="166" s="1" customFormat="1">
       <x:c r="B166" s="1" t="s">
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="C166" s="1" t="s">
         <x:v>429</x:v>
-      </x:c>
-      <x:c r="C166" s="1" t="s">
-        <x:v>430</x:v>
       </x:c>
       <x:c r="D166" s="1">
         <x:v>100</x:v>

</xml_diff>